<commit_message>
did data validation with the drop down and conditional highlighting and such
</commit_message>
<xml_diff>
--- a/product_report.xlsx
+++ b/product_report.xlsx
@@ -58,6 +58,16 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -656,7 +666,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>Invalid unit type : PCS; HSN code must be numeric: mm12</t>
+          <t>Invalid unit type : PCS</t>
         </is>
       </c>
     </row>
@@ -3347,6 +3357,19 @@
       <c r="AD34" t="inlineStr"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F1000">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(F2&lt;&gt;"", E2&lt;&gt;"", F2&lt;E2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="AA2:AA1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: pcs, doz, kgs, g, l, ml, d, mm, mo" type="list">
+      <formula1>"pcs,doz,kgs,g,l,ml,d,mm,mo"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid date order" error="End date cannot be earlier than Start date" type="custom">
+      <formula1>OR(E2="",F2&gt;=E2)</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10350,6 +10373,11 @@
       <c r="AE73" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="AC2:AC1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: GST_INTER, GST_INTRA, GST_EXPORT_LUT, GST_EXPORT_WP, GST_EXEMPT, GST_UT, NO_TAX" type="list">
+      <formula1>"GST_INTER,GST_INTRA,GST_EXPORT_LUT,GST_EXPORT_WP,GST_EXEMPT,GST_UT,NO_TAX"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10366,22 +10394,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>created_datetime_x</t>
+          <t>created_datetime</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>modified_datetime_x</t>
+          <t>modified_datetime</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>created_user_id_x</t>
+          <t>created_user_id</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>modified_user_id_x</t>
+          <t>modified_user_id</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -10411,22 +10439,22 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>created_datetime_y</t>
+          <t>created_datetime_master</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>modified_datetime_y</t>
+          <t>modified_datetime_master</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>created_user_id_y</t>
+          <t>created_user_id_master</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>modified_user_id_y</t>
+          <t>modified_user_id_master</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
@@ -17694,6 +17722,11 @@
       <c r="T85" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: textfield, date, phone number" type="list">
+      <formula1>"textfield,date,phone number"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>